<commit_message>
Update pipeline with new Pst genes and primers
</commit_message>
<xml_diff>
--- a/resources/fungicide_metadata.xlsx
+++ b/resources/fungicide_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vof23jop/Documents/JIC/Publications/1_MARPLE_stem_rust/Data/Pyproc_find-markers/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Diane-Saunders/loizos/MARPLE/PST/rebuild-MARPLE-PST/fix-marple-genes-Nov25/ new_pst_primers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{87C3F231-1D0C-934E-AA7B-055D19403102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E66C80D-47AD-DF42-98C1-AAA49058F500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="68640" yWindow="-1460" windowWidth="38400" windowHeight="21100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17500" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="variants" sheetId="3" r:id="rId3"/>
     <sheet name="var_seqs" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="131">
   <si>
     <t>Gene</t>
   </si>
@@ -424,12 +424,42 @@
   <si>
     <t>MASSLRPGLFSQVCAKPQTSQRMLSTSTTSTINRPLAQQVRPAFQRSVIQQSTRIAAFHATQRNSILPPLPQKIIGTANDPTPVPDPDYTHGSYHWSFERIVSAGLIPLTVAPFAAGSLNPVTDSILCALLVVHSHIGFESCIVDYFPKKRVPKTRAAAMWALRAGTVVLGLALYSFETNDVGITEAVARLWHA</t>
   </si>
+  <si>
+    <t>ATGTCTTCCCTGCTCAGCCCAGTTTTCGAGTTCATCGGCAGTTTCTCGTTGTTCGTTCAATTTACGATCTATCTCCTGCTCTCGATCGTCTCGATAGTCTCGATCAACATCTTCAACCAACTGGTAATCAGAGTCTGACTGCTCTCTTCTTTTTGAGCCAACGATCTGACTGTATCTGTCATCCTGTTTTTTGTTCTAGATTGTCCCCAAAAATGCGACCACTCCACCCGTCGTCTTCCACATATTCCCGATCATAGGCTCAGCAATCTCATACGGAATCGATCCATACGCTTTCCTAGAATCATGCAGAAAGAAATATGGGAACGTATTCACATTCATACTTATAAATAAGAAAGTGACTGTAGCTTTAGGTTTACAAGGAAACGCATTGGTTCTCAATGGGAAACTTGCTCAAGTTAATGCTGAAGAAGCCTATACCGCTCTCAGTATGTCATCTCATCTCTCGTCTTCTTCGCAATTTCCCTAAACTAATAATGAGTTCTTCTCCTTCTATTGAATTTTTCTACAGCTACTCCTGTATTCGGTACGGATGTAGTTTATGATGTCCCGAACGCAATCTTGATGCAACAAAAAAAATTCATCAAATCTGGCTTGACCACCGAAAACTTTCGTAAATACGTATCTACGATTGTCGATGAGACGATCGGTTATATCGAGGATCATATATTCCAGAGTAAGTTTGAGATTCTTTTATATCGACCATTCCCTCCCCCTTAACTTACTTGAGCATTTATCTCAGACCCAAAAACCCAGCAAGCTGTCAAAGATGCTCTCAAGGTGGCCTCAGAGATCACGATCTGTACCGCTTCGGCTACACTTCAAGGGCCTGAAGTCAGAGAAGGACTCAACACATCATTTGCGGATATATATCATGACTTAGATGGTGGATTTACACCCTTACATTTCGCTCTACCTGGACTACCTTTACCATCTTATCGAAAGAGAGATCTAGCACAAGTAGCCATGAGGAACTTCTATTTAAATATAATCAAAAAGAGAAGAGAAGATAACAGGGAAGGTCAATTAGGAGATATGATCGATAGTTTACAGGGACAAACTTATAAGGATGGTCGACCATTAACTGATAAAGAGATAGCACATATCATGATTGCACTTCTTATGGCCGGTCAACATACTAGTGCTGCCACTGGATCATGGTTAATCCTCCATCTAGCATCTCGTCCAGATCTTGTGAAGGAATTGAGGAAGGAACAGATCGAACTATTCGGTAAACCTGGTCAAACTGATGAGAACGAACTCGATCCTCTAGACCTTGAACGTGTTCAGAGTCCCTTGATGATTGCTTGTATCAAGGAGGTACTCAGACTTCATCCTCCGATCCATTCGATCATGCGAAAGGTACAGAGATCCTACTTCCTCTACACCTCACTTTATCAGATCGAAAAAAAAGCTGACCAGTCCATTTACATATATTTAGGTTAAATCGCCGATCACCGTACCACGAACATTGGCCTCTCTCAATGAAGATACGCCATACATAATCCCCTCGAGCCACTTTGTTTTAGCCGCACCAGGAACAGCACAACTCGATCCGAGCATCTGGACTGCACCGGATGAATTTGAACCTAGTAGATGGTTAAACCAACCTTCACCATTCAAGACCTCGACCACCACTACAAGTGGAGAAGAGAGCACCGCTCAAGAAGAGATGGTTGATTACGGGTTCGGTATGATTAGTAGTGGTGCTAATTCTCCCTTCTTACCTTTCGGAGCGGGCAGACATCGTTGTATTGGTGAACAATTCGCTTACATTCAATTATCTACTATCGGTGCTACCTTCATTCGTAATTGTGACATCGAATTAATCACTGATCAATTCCCTAAACCCGATTACACCGTACGTTTGTCTCTCTGTCGCTTTTTCTTTCTTTTTTTTTTTGGTTTCGATCCTTATCCTTTTTTTTTCTTTTTGCTTCGATGGTACTCATATTCGCTCATTTTTTTTTTTATTGATTTAGACTATGTTGGTTTGTCCACTCAAGCCCAGAGATATCAAATTTACCAGAAGAAATCATCTTTAA</t>
+  </si>
+  <si>
+    <t>Pst134EA_017948</t>
+  </si>
+  <si>
+    <t>ATGCTACGATCGAAAATACTCAACAGGATCAAGCCAGCGACTTCCAGCCTCAGCCTAGCCAAGCGAAGTTTTACGAGCAGCCCGTCATGCGCACGCATAATATCTAGTCAGCCAGTCAAAGCATCGGAGAGCAGCAGCATCGCATCCAAGTTCAGCAGTGGAAACTACCCGATCATCGACCACGAGTACGATGCTATCGTCGTCGGAGCTGGTGGGGCTGGCCTCAGAGCTGCATTCGGTTTAGCCGAAGCTGGGCTTAACACCGCTTGCATCACAAAATTATTCCCTACTCGTTCTCATACGGTGGCTGCTCAAGGCGGGGTCAATGCCGCACTGGGTAACATGACCGAGGTAAGTCACTGCCTCATCATCATCATCATCATCATCATCATCTGAAACTGATTGCTCTGGACATACTAGGACGATTGGCGTTGGCATATGTACGATACCGTCAAAGGATCGGATTGGTTGGGAGATCAAGATGCGATTCATTATATGTGCAAGGAAGCACCTCAAGCAGTAATCGAATTAGAACACTTTGGAGTCCCATTTTCGCGTACCAAGGAAGGGAAAATCTACCAAAGAGCCTTTGGTGGTCAATCCTTGAAATATGGAAAGGGAGGACAAGCTTATCGATGTGCAGCTGCAGCAGATCGAACCGGACATGCTATCCTACACACATTATATGGTCAATCATTACGACATAATACCAACTTCTTTGTCGAGTTTTTCGCACTAGATTTAATAATGGATGATTCGGGTAACTGTGTAGGAGTAACTGCCTATAACCAAGAAGATGGTACCCTACATCGATTCAGAGCTCATCAAACCGTCTTGGCTACCGGTGGTTATGGTCGGGCTTACTTCTCGTGTACTAGTGCTCATACTTGTTCTGGTGATGGTAACGCTATGGTCACCAGAGCTGGTTTACCTCTCCAAGATCTAGAATTCGTTCAGTTTCATCCAACCGGTATCTATGGTGCTGGTTGTTTGATCACCGAAGGATCAAGAGGAGAGGGTGGTTATCTATTAAACTCACAGGGAGAGAGATTTATGGTAAGTCCACTTTCACTGTCTCTATCTACCTCTCAACTAAAAGCGCTCTCTAATCTCGCTTTTTTCTATATCTTTCAAGGAACGATATGCGCCAACAGCTAAAGATCTAGCATCAAGAGACGTAGTCTCGAGATCGATGACCATCGAGATCAGAGAAGGTAGAGGAGTTGGACCGGATAAAGATCACTGTTACCTTCAACTCTCTCATCTACCTCCAGAAGTCCTCCACGAACGTCTCCCAGGTATCTCTGAAACTGCTGCCATCTTTGCCGGTGTTGATGTTACCAAGGAACCTGTAAGCTTCTTATTTTTCGACACCGCCTCTACCTCGATCATATCATTCTAATCACGTTCCTTCACCACTTTGTGTTGTCCGACGCGGTTTAGATTCCCGTTTTGCCAACTGTCAGTACGAGTTTCTCTATTTGAAGCACAACCTTTCTTTGAAATAATTAAATCGAGTGTTTCTAGGTACACTACAACATGGGAGGAATACCAACGAACTACCATGGTCAAGTGATAACGCAAGATCCAAAGACAGGAGGAGACAAGATAGTAGGAGGATTATATGCAGCGGGAGAAGCAGCATGTGTATCGGTACATGGAGCGAACAGATTAGGCGCGAATTCATTATTAGATATAGTAGTATTTGGAAGAGCTTGTGCTAAACATATTTCAGCTAATATGGAACCTGGCAAACCACATAAACCTATGCCTGAAGATGCCGGTATGAAATCCATCGAAGATTTGGACAAATTGAGGAACGCTAAGGGACCTAAACCTACCGCTCAAATTAGAAATGATATGCAAAGAGTTATGCAAAATGATGCCGCCGTCTTTAGAACTCAATCTTCTCTTGCTGAAGGCGTTACTAAAATTCATAAAGTCGTCGATTCTTTCAAAGATGTAGGTGTTACCGATAGAAGTATGATTTGGAATACGTTAGTTCATCTTCTTAAAACTCCCTTCCCTTGCCTTTTCTTTCCATCTGAACTATTGTGGTATGAAATCTAACGTATTTGTTTTCAATAAAACAGCGATTTGGTGGAGACTCTAGAGTTAAGAAATTTGTTGACTTGTGCTGCTCAAACTATGTCTTCAGCTGAAGCTAGAAAAGAATCAAGAGGAGCTCATGCACGTGAAGATTTCCCTGAACGAGAGGATGATACATGGATGAAACATACCGTCTGTCTTTCTTTTCTTCCCCCCTCTCTTTCTTTCTCTCCTTCAATGAATATTCAAATGATCGAGAAAAAACTGATCTTAGTGTTATTTGAATTTATTTATTTTTAGTTGTCTTGGCATAATCCTGAATCTGGTGATCCTGTTAAACTCACTTATCGGGACGTTATCAGTTCTACTTTAGATGAAAATGAATGCAAGAGGTTCGTCTCCTCTTTTTTCCTCAACCCCCCTTTATGACTTTTATTGACTTCATGTTTTTTTTTTTCCTTTTTTTTGCTTAGTGTTCCTCCTTTTAAACGTACTTATTGA</t>
+  </si>
+  <si>
+    <t>Pst134EA_002550</t>
+  </si>
+  <si>
+    <t>ATGTTAACCGTACAGAACATACTCAGACCATGTCTTCGATCCACTCAACTTCGAACAGCCACTTGCTCGGTAAGCTCTCAAAACAGCGAAGAAAGGGAGAGAGAGAGACTGACTGACATGTCTCTGGAATCCAGCTGTCCAACATCCGCTTGATATCATCAAGCAAGTCCACATCATTTGCCACACCAGCCGAGGAACATGCTGGACAACAATCGAGCACGGCGAATGAATCGAAGGAGTTCTCGATCTATCGATGGAACCCAGACGAACCCAGCAAGAAACCTAGTCTCCAAACTTACTCTATCGATCTCAAGAAATGCGGACCCATGGTGCTCGACGCTTTAATCAAGATCAAGAACGAAATCGATCCTACTCTCACGTTCAGAAGAAGTTGTAGAGAAGGTATCTGTGGTTCTTGCGCTATGAATATCGACGGAGTTAATACTTTGGCTTGTTTGAAACGTATCAATAAGGAAACTAGCGCTCCTGTTAAGATCTATCCTCTTCCCCACAGTAAGCTTTTCTCCCCTCCTCCTCCAAACATCACAAAAACAACTAAGAATCATTTTTTCTGTTATAAAGTGTACATCATTAAGGATCTTGTACCGGATATGACTCATTTCTATAAACAGTATAAATCTATCGAGCCTTTTTTGAAAAATGATAACCCTCCTGCCCAAGGTGAATTCTTACAATCTCCCGAAGATCGTAAGAAGCTTGATGGGATGTACGAGTGTATCTTATGTGCATGTTGCTGTGAGTTTTTTATTTATTTATTTATGAATATATCTTGTCCCCCAATGAAACTTAACGATTTGTCTGTCTTATCTATTAGCTACTAGTTGTCCTAGTTATTGGTGGAACCAAGACGAATACTTAGGACCAGCAGTTTTGATGCAAGCTTATCGGTAAGACCTCCCCTTAAAACAGATCGTCTGTATCTATTTCTTCACTGACTTTTTCTTTCGGGGACAATCATAGATGGATGGCCGATTCTCGTGATTCTTATGGCGAAGATCGTAAAGAGAAACTCCAGAATACTCTCTCCCTTTACAGATGTCACACCATCTTTAACTGTACTAAAACTTGTCCTAAGGGTTTGAACGTAAGTCGTGTCCCTTTTTTTTATGTCACAGGTAGTTTTACCAGTTACTGATAAATTGTTGCGTTTATTATTTGGACAGCCCGCTAAAGCTATTTCTCACATCAAACGTGAAATGGCAACTGCTTAA</t>
+  </si>
+  <si>
+    <t>Pst134EA_000043</t>
+  </si>
+  <si>
+    <t>ATGAGCTCATCGATACTCAAGCAGACCATTCTACGTACTCAGTCACTCATCCCACTCAATACAGTCAGACCATCGATCTTAGGGAGCTTATCAGGCTTGAAGCAACAGAGGTAAGATCGATCTCGTAATGATGTATCTAGAGATCTTCTGATCGCTCTTCGTTTGCTCAGATTCAATAGCACTAAAACACTGAAATGCTCAGAAGAGGATGCACTCAAGTTACTCAATCAACAACGAAAACTTCGTCCATCTTCTCCTCATTTCACTATCTACGAACCTCAGGTATTTTATTCTCTCGATCACTTGTACTTTCGAGAAAATTGACATCATGCTTGGTTTTCCTAGTTGACTTGGTACTCTAGTATCGCAAATCGAATCACTGGTTGCGGTTTATCATTAGGTTTAGTGCAAATCTCTCTCCCGAAGAGATCGATCATGAGAAATAAAACACGAACTTAACTGGTTTTTATACTGTTTTCTTTTTAGGTTTTTACGCGTATGCTTTAGGATATATGGCCTTACCTAATAGCATGCCATTAGATTCAGAAACTGTTGTACAATTTGTCGCTTCTAGTCCTGAATGGGCTAAGGTAAAACATATATCCTTCTCAATTCATATCTAGATCGCTTACTTGAACTTGATTTCTCTTTCGGTTTGTTTGTTTAATAGGTTGCCGGAAAAGCTGTTGTAGCTTTACCATTCACTTATCATACTTTCAACGGAGTCAGACATTTAGCTTGGGACATGGGATACCGTAAGATCACTTTCCAAAAAAGAATCTTATATAATATTGGGAAATAACTAACTTCTTAATCTCCGTTTACTTATCAATGTAGTACTTGATCTCAAAACAAGTTACACCGCAGGTAAACCAGAACCTCCATCAATTCCTAAATGCATGTAACAAAACTGATGTAATATGTATCATTTATAGGTTACACCGTCCTTGGTTTAACCGCAGTTTCGACCGTTGGATTAGTTCTCATCTAA</t>
+  </si>
+  <si>
+    <t>Pst134EA_032255</t>
+  </si>
+  <si>
+    <t>ATGTCTCAGACCAATCGAATTATCATGTCCGCCAGTCGAATGTGCCCAACGACACGCAGCATGACCAACAATCTCAATCTGAATCGAATTTCGTTTATGGTCCCTCAATACCATCGATTGTCGACCAGTACGTCATCATAACTCTTTCGATTAGCATCATGGCTATCTTTAGTGCATACTGTTGACTTCAAGCTTGACATGAATATCTAGGCTCGACTTCCCTTGCAAAATCCACTCCGATCGTCAAAGCAAACTCGACTGCAGATGCCCGTAAGTACCACCACGATCATGCCTTGCACCACTTCAGTCGCGAAGAATCACACGTACTGATGGATTCCGCTTGTTCTCAATTTAAGCCTACGTTAAAGGTACGATTAACGACCCCACTACCTTCCCACCCCCAAGCAAAGCCCATGGATCGATACATTGGACTTTCGAAAGATCCGTCGCTGCCAGTTTGATCCCGCTCTCGGCCGCTACTGCTATCTCTAGTGCCAACCCTATACTTGACGGAGTCATCGGAGTTTTCCTGATCGCCCATTCCCACATGGTTTGTCCCTCTAGGATGGATGCCTTCGCTGAATCTGATAACCTGATCACAGTATCGACTAAAGCTGAACTTTAACCCCTCTTTATCGCCTTTCTGTTAAAAAACTACGTTGATAGGGATTCGATCAAGCTTTAGTGGATTACGTTCCCAAACGTAAATTTCCTGTAATAAGTCCTATCGCCACTTGGACTTTACGCGCGCTTACTTGTGGTGTCCTAGTTGGGGTGTACCAATTCAACACTCATGATATCGGTCAGTACTTCTTCAGGTCGCTCATATCTCCTTGTCTGAGTCCGATTGCCCTGACCACACTGCCAACCACCACCTTTCCTTCCTGATATTTCTTCATTGTGGGTAGGTATGACCGAGTTAATCAAGAAAGCGTGGAAGGCATGA</t>
+  </si>
+  <si>
+    <t>Pst134EA_005128</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -475,13 +505,55 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="5"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="12">
@@ -614,38 +686,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -673,7 +744,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -684,7 +755,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -710,6 +780,60 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -918,25 +1042,25 @@
       <c r="A3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="4">
         <v>107</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="13" t="s">
+      <c r="F3" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="12" t="s">
         <v>16</v>
       </c>
     </row>
@@ -944,25 +1068,25 @@
       <c r="A4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="4">
         <v>134</v>
       </c>
-      <c r="C4" s="11">
+      <c r="C4" s="4">
         <v>131</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="13" t="s">
+      <c r="F4" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="12" t="s">
         <v>16</v>
       </c>
     </row>
@@ -970,25 +1094,25 @@
       <c r="A5" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="4">
         <v>136</v>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="4">
         <v>133</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="13" t="s">
+      <c r="F5" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="12" t="s">
         <v>19</v>
       </c>
     </row>
@@ -996,25 +1120,25 @@
       <c r="A6" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="4">
         <v>137</v>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="4">
         <v>134</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="13" t="s">
+      <c r="F6" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="12" t="s">
         <v>103</v>
       </c>
     </row>
@@ -1022,25 +1146,25 @@
       <c r="A7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="4">
         <v>145</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="4">
         <v>142</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" s="13" t="s">
+      <c r="F7" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1048,25 +1172,25 @@
       <c r="A8" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="4">
         <v>178</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H8" s="13" t="s">
+      <c r="F8" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1074,25 +1198,25 @@
       <c r="A9" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="4">
         <v>188</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" s="13" t="s">
+      <c r="F9" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="12" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1100,25 +1224,25 @@
       <c r="A10" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="4">
         <v>208</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="4">
         <v>204</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="13" t="s">
+      <c r="F10" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1126,25 +1250,25 @@
       <c r="A11" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="4">
         <v>284</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="4">
         <v>280</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H11" s="13" t="s">
+      <c r="F11" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1152,25 +1276,25 @@
       <c r="A12" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="4">
         <v>303</v>
       </c>
-      <c r="C12" s="11">
+      <c r="C12" s="4">
         <v>299</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H12" s="13" t="s">
+      <c r="F12" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="12" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1178,25 +1302,25 @@
       <c r="A13" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="4">
         <v>311</v>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="4">
         <v>307</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H13" s="13" t="s">
+      <c r="F13" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1204,25 +1328,25 @@
       <c r="A14" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="4">
         <v>312</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C14" s="4">
         <v>308</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F14" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H14" s="13" t="s">
+      <c r="F14" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1230,25 +1354,25 @@
       <c r="A15" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="4">
         <v>379</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H15" s="13" t="s">
+      <c r="F15" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="12" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1256,25 +1380,25 @@
       <c r="A16" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="4">
         <v>381</v>
       </c>
-      <c r="C16" s="11">
+      <c r="C16" s="4">
         <v>379</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F16" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H16" s="13" t="s">
+      <c r="F16" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H16" s="12" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1282,25 +1406,25 @@
       <c r="A17" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="4">
         <v>410</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="4">
         <v>416</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F17" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H17" s="13" t="s">
+      <c r="F17" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1308,25 +1432,25 @@
       <c r="A18" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="4">
         <v>412</v>
       </c>
-      <c r="C18" s="11">
+      <c r="C18" s="4">
         <v>418</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="D18" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F18" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H18" s="13" t="s">
+      <c r="F18" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1334,25 +1458,25 @@
       <c r="A19" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="4">
         <v>459</v>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="4">
         <v>466</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F19" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H19" s="13" t="s">
+      <c r="F19" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="12" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1360,25 +1484,25 @@
       <c r="A20" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="4">
         <v>460</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="4">
         <v>467</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="F20" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H20" s="13" t="s">
+      <c r="F20" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" s="12" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1386,25 +1510,25 @@
       <c r="A21" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="4">
         <v>461</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="4">
         <v>468</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E21" s="11" t="s">
+      <c r="E21" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F21" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G21" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H21" s="13" t="s">
+      <c r="F21" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21" s="12" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1412,25 +1536,25 @@
       <c r="A22" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="4">
         <v>490</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="4">
         <v>469</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="E22" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F22" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G22" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H22" s="13" t="s">
+      <c r="F22" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="12" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1438,25 +1562,25 @@
       <c r="A23" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="4">
         <v>510</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D23" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E23" s="11" t="s">
+      <c r="E23" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F23" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G23" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H23" s="13" t="s">
+      <c r="F23" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23" s="12" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1464,25 +1588,25 @@
       <c r="A24" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="4">
         <v>513</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="D24" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E24" s="11" t="s">
+      <c r="E24" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F24" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G24" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H24" s="13" t="s">
+      <c r="F24" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H24" s="12" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1490,25 +1614,25 @@
       <c r="A25" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="4">
         <v>524</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E25" s="11" t="s">
+      <c r="E25" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F25" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G25" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H25" s="13" t="s">
+      <c r="F25" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" s="12" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1516,25 +1640,25 @@
       <c r="A26" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="4">
         <v>134</v>
       </c>
-      <c r="C26" s="11">
+      <c r="C26" s="4">
         <v>134</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="D26" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E26" s="11" t="s">
+      <c r="E26" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="12" t="s">
+      <c r="F26" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="G26" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H26" s="13" t="s">
+      <c r="G26" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" s="12" t="s">
         <v>109</v>
       </c>
     </row>
@@ -1542,25 +1666,25 @@
       <c r="A27" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="4">
         <v>79</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="4">
         <v>76</v>
       </c>
-      <c r="D27" s="11" t="s">
+      <c r="D27" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E27" s="11" t="s">
+      <c r="E27" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F27" s="14" t="s">
+      <c r="F27" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="G27" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H27" s="13" t="s">
+      <c r="G27" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H27" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1568,56 +1692,56 @@
       <c r="A28" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="11">
+      <c r="B28" s="4">
         <v>136</v>
       </c>
-      <c r="C28" s="11">
+      <c r="C28" s="4">
         <v>134</v>
       </c>
-      <c r="D28" s="11" t="s">
+      <c r="D28" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E28" s="11" t="s">
+      <c r="E28" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F28" s="14" t="s">
+      <c r="F28" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="G28" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H28" s="13" t="s">
+      <c r="G28" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H28" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="B29" s="16">
+      <c r="A29" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B29" s="15">
         <v>175</v>
       </c>
-      <c r="C29" s="16" t="s">
+      <c r="C29" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D29" s="16" t="s">
+      <c r="D29" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="E29" s="16" t="s">
+      <c r="E29" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="F29" s="17" t="s">
+      <c r="F29" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="G29" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="H29" s="18" t="s">
+      <c r="G29" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H29" s="17" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" s="19" t="s">
+      <c r="A30" s="18" t="s">
         <v>35</v>
       </c>
       <c r="B30" s="7">
@@ -1638,246 +1762,246 @@
       <c r="G30" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="20" t="s">
+      <c r="H30" s="19" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" s="21" t="s">
+      <c r="A31" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="4">
         <v>225</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="4">
         <v>217</v>
       </c>
-      <c r="D31" s="11" t="s">
+      <c r="D31" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E31" s="11" t="s">
+      <c r="E31" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F31" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G31" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H31" s="13" t="s">
+      <c r="F31" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" s="12" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="21" t="s">
+      <c r="A32" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="11">
+      <c r="B32" s="4">
         <v>265</v>
       </c>
-      <c r="C32" s="11">
+      <c r="C32" s="4">
         <v>257</v>
       </c>
-      <c r="D32" s="11" t="s">
+      <c r="D32" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E32" s="11" t="s">
+      <c r="E32" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F32" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G32" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H32" s="13" t="s">
+      <c r="F32" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H32" s="12" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="21" t="s">
+      <c r="A33" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="11">
+      <c r="B33" s="4">
         <v>267</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33" s="4">
         <v>259</v>
       </c>
-      <c r="D33" s="11" t="s">
+      <c r="D33" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E33" s="11" t="s">
+      <c r="E33" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F33" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G33" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H33" s="13" t="s">
+      <c r="F33" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H33" s="12" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="21" t="s">
+      <c r="A34" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B34" s="11">
+      <c r="B34" s="4">
         <v>268</v>
       </c>
-      <c r="C34" s="11">
+      <c r="C34" s="4">
         <v>260</v>
       </c>
-      <c r="D34" s="11" t="s">
+      <c r="D34" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E34" s="11" t="s">
+      <c r="E34" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="F34" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G34" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H34" s="22" t="s">
+      <c r="F34" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H34" s="21" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B35" s="11">
+      <c r="B35" s="4">
         <v>269</v>
       </c>
-      <c r="C35" s="11">
+      <c r="C35" s="4">
         <v>261</v>
       </c>
-      <c r="D35" s="11" t="s">
+      <c r="D35" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E35" s="11" t="s">
+      <c r="E35" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F35" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G35" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H35" s="13" t="s">
+      <c r="F35" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H35" s="12" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" s="21" t="s">
+      <c r="A36" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="11">
+      <c r="B36" s="4">
         <v>276</v>
       </c>
-      <c r="C36" s="11">
+      <c r="C36" s="4">
         <v>268</v>
       </c>
-      <c r="D36" s="11" t="s">
+      <c r="D36" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E36" s="11" t="s">
+      <c r="E36" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F36" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G36" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H36" s="13" t="s">
+      <c r="F36" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H36" s="12" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" s="21" t="s">
+      <c r="A37" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="4">
         <v>277</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D37" s="11" t="s">
+      <c r="D37" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E37" s="11" t="s">
+      <c r="E37" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F37" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G37" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H37" s="13" t="s">
+      <c r="F37" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H37" s="12" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A38" s="23" t="s">
+      <c r="A38" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="B38" s="16">
+      <c r="B38" s="15">
         <v>227</v>
       </c>
-      <c r="C38" s="16" t="s">
+      <c r="C38" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D38" s="16" t="s">
+      <c r="D38" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E38" s="16" t="s">
+      <c r="E38" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="F38" s="24" t="s">
+      <c r="F38" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="G38" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="H38" s="18" t="s">
+      <c r="G38" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H38" s="17" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A39" s="25" t="s">
+      <c r="A39" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B39" s="26">
+      <c r="B39" s="25">
         <v>86</v>
       </c>
-      <c r="C39" s="26">
-        <v>85</v>
-      </c>
-      <c r="D39" s="26" t="s">
+      <c r="C39" s="25">
+        <v>81</v>
+      </c>
+      <c r="D39" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="E39" s="26" t="s">
+      <c r="E39" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="F39" s="27" t="s">
+      <c r="F39" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="G39" s="26" t="s">
-        <v>13</v>
-      </c>
-      <c r="H39" s="28" t="s">
+      <c r="G39" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="H39" s="27" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" s="19" t="s">
+      <c r="A40" s="18" t="s">
         <v>47</v>
       </c>
       <c r="B40" s="7">
@@ -1903,210 +2027,210 @@
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41" s="21" t="s">
+      <c r="A41" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B41" s="11">
+      <c r="B41" s="4">
         <v>50</v>
       </c>
-      <c r="C41" s="11">
+      <c r="C41" s="4">
         <v>63</v>
       </c>
-      <c r="D41" s="11" t="s">
+      <c r="D41" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E41" s="11" t="s">
+      <c r="E41" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F41" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G41" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H41" s="13" t="s">
+      <c r="F41" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H41" s="12" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" s="21" t="s">
+      <c r="A42" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B42" s="11">
+      <c r="B42" s="4">
         <v>114</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D42" s="11" t="s">
+      <c r="D42" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E42" s="11" t="s">
+      <c r="E42" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F42" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G42" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H42" s="13" t="s">
+      <c r="F42" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H42" s="12" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" s="21" t="s">
+      <c r="A43" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B43" s="11">
+      <c r="B43" s="4">
         <v>129</v>
       </c>
-      <c r="C43" s="11">
+      <c r="C43" s="4">
         <v>135</v>
       </c>
-      <c r="D43" s="11" t="s">
+      <c r="D43" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E43" s="11" t="s">
+      <c r="E43" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="F43" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G43" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H43" s="13" t="s">
+      <c r="F43" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H43" s="12" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A44" s="21" t="s">
+      <c r="A44" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B44" s="11">
+      <c r="B44" s="4">
         <v>124</v>
       </c>
-      <c r="C44" s="11">
+      <c r="C44" s="4">
         <v>114</v>
       </c>
-      <c r="D44" s="11" t="s">
+      <c r="D44" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E44" s="11" t="s">
+      <c r="E44" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F44" s="12" t="s">
+      <c r="F44" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G44" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H44" s="13" t="s">
+      <c r="G44" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H44" s="12" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A45" s="21" t="s">
+      <c r="A45" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B45" s="11">
+      <c r="B45" s="4">
         <v>134</v>
       </c>
-      <c r="C45" s="11">
+      <c r="C45" s="4">
         <v>124</v>
       </c>
-      <c r="D45" s="11" t="s">
+      <c r="D45" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E45" s="11" t="s">
+      <c r="E45" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F45" s="12" t="s">
+      <c r="F45" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G45" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H45" s="13" t="s">
+      <c r="G45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H45" s="12" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A46" s="21" t="s">
+      <c r="A46" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B46" s="11">
+      <c r="B46" s="4">
         <v>138</v>
       </c>
-      <c r="C46" s="11" t="s">
+      <c r="C46" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D46" s="11" t="s">
+      <c r="D46" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E46" s="11" t="s">
+      <c r="E46" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F46" s="12" t="s">
+      <c r="F46" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G46" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H46" s="13" t="s">
+      <c r="G46" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H46" s="12" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A47" s="21" t="s">
+      <c r="A47" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B47" s="11">
+      <c r="B47" s="4">
         <v>145</v>
       </c>
-      <c r="C47" s="11">
+      <c r="C47" s="4">
         <v>135</v>
       </c>
-      <c r="D47" s="11" t="s">
+      <c r="D47" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E47" s="11" t="s">
+      <c r="E47" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="F47" s="12" t="s">
+      <c r="F47" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G47" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H47" s="13" t="s">
+      <c r="G47" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H47" s="12" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A48" s="23" t="s">
+      <c r="A48" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="B48" s="16">
+      <c r="B48" s="15">
         <v>178</v>
       </c>
-      <c r="C48" s="16" t="s">
+      <c r="C48" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D48" s="16" t="s">
+      <c r="D48" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="E48" s="16" t="s">
+      <c r="E48" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="F48" s="24" t="s">
+      <c r="F48" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="G48" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="H48" s="18" t="s">
+      <c r="G48" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H48" s="17" t="s">
         <v>113</v>
       </c>
     </row>
@@ -2146,130 +2270,130 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="C1" s="30" t="s">
+      <c r="C1" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="D1" s="30" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2" s="32" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="33" t="s">
+      <c r="A2" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="D2" s="32" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="32" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="33" t="s">
+      <c r="A3" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="32" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="35" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="36" t="s">
+      <c r="A4" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="36" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="39"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="37"/>
     </row>
     <row r="6" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="39" t="s">
         <v>60</v>
       </c>
-      <c r="C6" s="41" t="s">
+      <c r="C6" s="39" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="42" t="s">
+      <c r="D6" s="40" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="34" t="s">
         <v>117</v>
       </c>
-      <c r="C7" s="36" t="s">
+      <c r="C7" s="34" t="s">
         <v>119</v>
       </c>
-      <c r="D7" s="37" t="s">
+      <c r="D7" s="35" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="43"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="41"/>
     </row>
     <row r="9" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="D9" s="34" t="s">
+      <c r="D9" s="32" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="35" t="s">
+      <c r="A10" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="34" t="s">
         <v>120</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="C10" s="34" t="s">
         <v>119</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="D10" s="35" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2289,166 +2413,166 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="30" t="s">
+      <c r="C1" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="30" t="s">
+      <c r="D1" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="E1" s="31" t="s">
+      <c r="E1" s="30" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="32" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="33" t="s">
+      <c r="A2" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="33"/>
-      <c r="E2" s="44">
+      <c r="D2" s="3"/>
+      <c r="E2" s="42">
         <v>510</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="32" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="33" t="s">
+      <c r="A3" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="33"/>
-      <c r="E3" s="44">
+      <c r="D3" s="3"/>
+      <c r="E3" s="42">
         <v>525</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="35" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="36" t="s">
+      <c r="A4" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="36"/>
-      <c r="E4" s="45">
+      <c r="D4" s="34"/>
+      <c r="E4" s="43">
         <v>537</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="31"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="30"/>
     </row>
     <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="30"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="31"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="30"/>
     </row>
     <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="29" t="s">
+      <c r="A7" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="30"/>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="31"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="30"/>
     </row>
     <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="40" t="s">
+      <c r="A8" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="41" t="s">
+      <c r="C8" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="41"/>
-      <c r="E8" s="46">
+      <c r="D8" s="39"/>
+      <c r="E8" s="44">
         <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="33"/>
-      <c r="E9" s="44">
+      <c r="D9" s="3"/>
+      <c r="E9" s="42">
         <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="33"/>
-      <c r="E10" s="44">
+      <c r="D10" s="3"/>
+      <c r="E10" s="42">
         <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="C11" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="33"/>
-      <c r="E11" s="44">
+      <c r="D11" s="3"/>
+      <c r="E11" s="42">
         <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12" s="35" t="s">
+      <c r="A12" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="36" t="s">
+      <c r="B12" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="36" t="s">
+      <c r="C12" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="36"/>
-      <c r="E12" s="45">
+      <c r="D12" s="34"/>
+      <c r="E12" s="43">
         <v>190</v>
       </c>
     </row>
@@ -2464,145 +2588,209 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.1640625" style="3"/>
-    <col min="2" max="2" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.1640625" style="3"/>
+    <col min="2" max="2" width="18.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="255.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.1640625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="30" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="32" t="s">
+    <row r="2" spans="1:3" s="69" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="68" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="69" t="s">
         <v>70</v>
       </c>
-      <c r="C2" s="44" t="s">
+      <c r="C2" s="70" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="35" t="s">
+    <row r="3" spans="1:3" s="69" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="71" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="72" t="s">
         <v>73</v>
       </c>
-      <c r="C3" s="45" t="s">
+      <c r="C3" s="73" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="40" t="s">
+    <row r="4" spans="1:3" s="64" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="62" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="63" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="35" t="s">
+    <row r="5" spans="1:3" s="64" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="65" t="s">
         <v>78</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="66" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="45" t="s">
+      <c r="C5" s="67" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="40" t="s">
+    <row r="6" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="56" t="s">
         <v>82</v>
       </c>
-      <c r="C6" s="46" t="s">
+      <c r="C6" s="57" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="35" t="s">
+    <row r="7" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="58" t="s">
         <v>84</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="59" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="45" t="s">
+      <c r="C7" s="60" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="40" t="s">
+    <row r="8" spans="1:3" s="48" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="45" t="s">
         <v>87</v>
       </c>
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="C8" s="46" t="s">
+      <c r="C8" s="47" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="32" t="s">
+    <row r="9" spans="1:3" s="48" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="49" t="s">
         <v>90</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="48" t="s">
         <v>91</v>
       </c>
-      <c r="C9" s="44" t="s">
+      <c r="C9" s="50" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="35" t="s">
+    <row r="10" spans="1:3" s="48" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="51" t="s">
         <v>93</v>
       </c>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="52" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="45" t="s">
+      <c r="C10" s="53" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="40" t="s">
+    <row r="11" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="74" t="s">
         <v>96</v>
       </c>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="75" t="s">
         <v>97</v>
       </c>
-      <c r="C11" s="46" t="s">
+      <c r="C11" s="76" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="35" t="s">
+    <row r="12" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="78" t="s">
         <v>99</v>
       </c>
-      <c r="B12" s="36" t="s">
+      <c r="B12" s="79" t="s">
         <v>100</v>
       </c>
-      <c r="C12" s="45" t="s">
+      <c r="C12" s="80" t="s">
         <v>101</v>
       </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="98"/>
+      <c r="B13" s="98"/>
+      <c r="C13" s="98"/>
+    </row>
+    <row r="14" spans="1:3" s="69" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="87" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="92" t="s">
+        <v>122</v>
+      </c>
+      <c r="C14" s="82" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" s="64" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="88" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="93" t="s">
+        <v>124</v>
+      </c>
+      <c r="C15" s="83" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="89" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="94" t="s">
+        <v>126</v>
+      </c>
+      <c r="C16" s="84" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" s="81" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="90" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="95" t="s">
+        <v>128</v>
+      </c>
+      <c r="C17" s="85" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" s="77" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="91" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="96" t="s">
+        <v>130</v>
+      </c>
+      <c r="C18" s="86" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B19" s="97"/>
     </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>

</xml_diff>

<commit_message>
Added Cob fungicide checks for Pst
</commit_message>
<xml_diff>
--- a/resources/fungicide_metadata.xlsx
+++ b/resources/fungicide_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vof23jop/Documents/JIC/Publications/1_MARPLE_stem_rust/Data/Pyproc_find-markers/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vof23jop/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{87C3F231-1D0C-934E-AA7B-055D19403102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40698CFD-830B-B742-A956-DDAB4CAE0823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="68640" yWindow="-1460" windowWidth="38400" windowHeight="21100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17660" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="123">
   <si>
     <t>Gene</t>
   </si>
@@ -423,6 +423,12 @@
   </si>
   <si>
     <t>MASSLRPGLFSQVCAKPQTSQRMLSTSTTSTINRPLAQQVRPAFQRSVIQQSTRIAAFHATQRNSILPPLPQKIIGTANDPTPVPDPDYTHGSYHWSFERIVSAGLIPLTVAPFAAGSLNPVTDSILCALLVVHSHIGFESCIVDYFPKKRVPKTRAAAMWALRAGTVVLGLALYSFETNDVGITEAVARLWHA</t>
+  </si>
+  <si>
+    <t>Cob</t>
+  </si>
+  <si>
+    <t>ATGAGAATTCTAAAGACGCATCCGATTCTAGGTCTAGTTAATTCTTATATAGGGGATTCACCACAACCAGCCAATATTAGTTATATATGGAACTTTGGAAGTCTTCTAGGATGTTGTCTTATCATTCAGATTATTACAGGAGTAACTCTAGCGATGCATTATACACCAAGTGTTGATCTAGCCTTTATTTCAGTGGAGCATATCATAAGAGATGTTGAATATGGTTGACTGATTAGGTATCTTCACGCTAATGTAGCTTCTTTTTTTTTCATTTTTGTATATATACACATTGGAAGAGGGCTATACTACGGTTCTTACAAGTCACCAAGGACACTTCTATGAGCCATTGGTGTAATTATTCTAATTGTTATAATAGCGACAGCCTTTATGGGATACGTTCTACCTTACGGACAGATGTCACTATGAGGTATAATTACGAATCTAATAAGTGCAATTCCATGAGTGGGTGGGGATCTTGTTGAATTTATTTGAGGAGGGTTTAGTGTTAACAATGCGACTCTGAACAGATTTTTTAGTCTTCATTTTGTACTACCTTTCATTCTTGCTGCACTTGTTGTAATACATCTTCTCACGCTTCATGAGCATGGTTCTAATAATCCTCTTGGGGTTTCAGGGAATGCGGATAGGCTGCCAATGGCTCCTAATTATATTTTCAAGGACCTAGTTACCATTTTCCTTTTCCTTCTTGTTCTTGCTATGTTCGTAATGTATGCACCAAACATAATAGGGCATTCTGATAATTATATCCCAGCTAATCCGATACAGACACCAGCTTCGATTGATTGATATCTTCTTCCATTCTATGCTATTCTACGTTCTATTCCTAATAAACTACTAGGGGTGATAGCCATGTTTGCAAGTCTTCTAATCCTGCTTGCCATACCGGTAATAGACCGGAGTCGAATGAGAGGGAGTCAATTTAGACCTCTAAATAGATTAATATTCTGAGTTCTGGTAGCGGATTTTCTAGTACTCATGTACCTAGGTTCTCAACATGTTGAGCAACCTTATATTCTTGTTGGTCAAATTGCAACAGCACTCTATTTTGCATGATTTGTTGTACTTATTCCGCTAACCTCAATCATTGAAAATACTCTAATGGATCTTAATGATGATAAGATTTAG</t>
   </si>
 </sst>
 </file>
@@ -614,38 +620,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -673,7 +678,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -684,7 +689,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -710,6 +714,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -918,25 +925,25 @@
       <c r="A3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="4">
         <v>107</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="13" t="s">
+      <c r="F3" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="12" t="s">
         <v>16</v>
       </c>
     </row>
@@ -944,25 +951,25 @@
       <c r="A4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="4">
         <v>134</v>
       </c>
-      <c r="C4" s="11">
+      <c r="C4" s="4">
         <v>131</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="13" t="s">
+      <c r="F4" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="12" t="s">
         <v>16</v>
       </c>
     </row>
@@ -970,25 +977,25 @@
       <c r="A5" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="4">
         <v>136</v>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="4">
         <v>133</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="13" t="s">
+      <c r="F5" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="12" t="s">
         <v>19</v>
       </c>
     </row>
@@ -996,25 +1003,25 @@
       <c r="A6" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="4">
         <v>137</v>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="4">
         <v>134</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="13" t="s">
+      <c r="F6" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="12" t="s">
         <v>103</v>
       </c>
     </row>
@@ -1022,25 +1029,25 @@
       <c r="A7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="4">
         <v>145</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="4">
         <v>142</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" s="13" t="s">
+      <c r="F7" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1048,25 +1055,25 @@
       <c r="A8" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="4">
         <v>178</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H8" s="13" t="s">
+      <c r="F8" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1074,25 +1081,25 @@
       <c r="A9" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="4">
         <v>188</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" s="13" t="s">
+      <c r="F9" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="12" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1100,25 +1107,25 @@
       <c r="A10" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="4">
         <v>208</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="4">
         <v>204</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="13" t="s">
+      <c r="F10" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1126,25 +1133,25 @@
       <c r="A11" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="4">
         <v>284</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="4">
         <v>280</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H11" s="13" t="s">
+      <c r="F11" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1152,25 +1159,25 @@
       <c r="A12" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="4">
         <v>303</v>
       </c>
-      <c r="C12" s="11">
+      <c r="C12" s="4">
         <v>299</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H12" s="13" t="s">
+      <c r="F12" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="12" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1178,25 +1185,25 @@
       <c r="A13" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="4">
         <v>311</v>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="4">
         <v>307</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H13" s="13" t="s">
+      <c r="F13" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1204,25 +1211,25 @@
       <c r="A14" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="4">
         <v>312</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C14" s="4">
         <v>308</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F14" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H14" s="13" t="s">
+      <c r="F14" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1230,25 +1237,25 @@
       <c r="A15" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="4">
         <v>379</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H15" s="13" t="s">
+      <c r="F15" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="12" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1256,25 +1263,25 @@
       <c r="A16" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="4">
         <v>381</v>
       </c>
-      <c r="C16" s="11">
+      <c r="C16" s="4">
         <v>379</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F16" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H16" s="13" t="s">
+      <c r="F16" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H16" s="12" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1282,25 +1289,25 @@
       <c r="A17" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="4">
         <v>410</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="4">
         <v>416</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F17" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H17" s="13" t="s">
+      <c r="F17" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1308,25 +1315,25 @@
       <c r="A18" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="4">
         <v>412</v>
       </c>
-      <c r="C18" s="11">
+      <c r="C18" s="4">
         <v>418</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="D18" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F18" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H18" s="13" t="s">
+      <c r="F18" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1334,25 +1341,25 @@
       <c r="A19" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="4">
         <v>459</v>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="4">
         <v>466</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F19" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H19" s="13" t="s">
+      <c r="F19" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="12" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1360,25 +1367,25 @@
       <c r="A20" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="4">
         <v>460</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="4">
         <v>467</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="F20" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H20" s="13" t="s">
+      <c r="F20" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" s="12" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1386,25 +1393,25 @@
       <c r="A21" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="4">
         <v>461</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="4">
         <v>468</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E21" s="11" t="s">
+      <c r="E21" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F21" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G21" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H21" s="13" t="s">
+      <c r="F21" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21" s="12" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1412,25 +1419,25 @@
       <c r="A22" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="4">
         <v>490</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="4">
         <v>469</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="E22" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F22" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G22" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H22" s="13" t="s">
+      <c r="F22" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="12" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1438,25 +1445,25 @@
       <c r="A23" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="4">
         <v>510</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D23" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E23" s="11" t="s">
+      <c r="E23" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F23" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G23" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H23" s="13" t="s">
+      <c r="F23" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23" s="12" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1464,25 +1471,25 @@
       <c r="A24" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="4">
         <v>513</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="D24" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E24" s="11" t="s">
+      <c r="E24" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F24" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G24" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H24" s="13" t="s">
+      <c r="F24" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H24" s="12" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1490,25 +1497,25 @@
       <c r="A25" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="4">
         <v>524</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E25" s="11" t="s">
+      <c r="E25" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F25" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G25" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H25" s="13" t="s">
+      <c r="F25" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" s="12" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1516,25 +1523,25 @@
       <c r="A26" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="4">
         <v>134</v>
       </c>
-      <c r="C26" s="11">
+      <c r="C26" s="4">
         <v>134</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="D26" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E26" s="11" t="s">
+      <c r="E26" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="12" t="s">
+      <c r="F26" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="G26" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H26" s="13" t="s">
+      <c r="G26" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" s="12" t="s">
         <v>109</v>
       </c>
     </row>
@@ -1542,25 +1549,25 @@
       <c r="A27" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="4">
         <v>79</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="4">
         <v>76</v>
       </c>
-      <c r="D27" s="11" t="s">
+      <c r="D27" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E27" s="11" t="s">
+      <c r="E27" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F27" s="14" t="s">
+      <c r="F27" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="G27" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H27" s="13" t="s">
+      <c r="G27" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H27" s="12" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1568,56 +1575,56 @@
       <c r="A28" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="11">
+      <c r="B28" s="4">
         <v>136</v>
       </c>
-      <c r="C28" s="11">
+      <c r="C28" s="4">
         <v>134</v>
       </c>
-      <c r="D28" s="11" t="s">
+      <c r="D28" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E28" s="11" t="s">
+      <c r="E28" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F28" s="14" t="s">
+      <c r="F28" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="G28" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H28" s="13" t="s">
+      <c r="G28" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H28" s="12" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="B29" s="16">
+      <c r="A29" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B29" s="15">
         <v>175</v>
       </c>
-      <c r="C29" s="16" t="s">
+      <c r="C29" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D29" s="16" t="s">
+      <c r="D29" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="E29" s="16" t="s">
+      <c r="E29" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="F29" s="17" t="s">
+      <c r="F29" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="G29" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="H29" s="18" t="s">
+      <c r="G29" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H29" s="17" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" s="19" t="s">
+      <c r="A30" s="18" t="s">
         <v>35</v>
       </c>
       <c r="B30" s="7">
@@ -1638,246 +1645,246 @@
       <c r="G30" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="20" t="s">
+      <c r="H30" s="19" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" s="21" t="s">
+      <c r="A31" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="4">
         <v>225</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="4">
         <v>217</v>
       </c>
-      <c r="D31" s="11" t="s">
+      <c r="D31" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E31" s="11" t="s">
+      <c r="E31" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F31" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G31" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H31" s="13" t="s">
+      <c r="F31" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" s="12" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="21" t="s">
+      <c r="A32" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="11">
+      <c r="B32" s="4">
         <v>265</v>
       </c>
-      <c r="C32" s="11">
+      <c r="C32" s="4">
         <v>257</v>
       </c>
-      <c r="D32" s="11" t="s">
+      <c r="D32" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E32" s="11" t="s">
+      <c r="E32" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F32" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G32" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H32" s="13" t="s">
+      <c r="F32" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H32" s="12" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="21" t="s">
+      <c r="A33" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="11">
+      <c r="B33" s="4">
         <v>267</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33" s="4">
         <v>259</v>
       </c>
-      <c r="D33" s="11" t="s">
+      <c r="D33" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E33" s="11" t="s">
+      <c r="E33" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F33" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G33" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H33" s="13" t="s">
+      <c r="F33" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H33" s="12" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="21" t="s">
+      <c r="A34" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B34" s="11">
+      <c r="B34" s="4">
         <v>268</v>
       </c>
-      <c r="C34" s="11">
+      <c r="C34" s="4">
         <v>260</v>
       </c>
-      <c r="D34" s="11" t="s">
+      <c r="D34" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E34" s="11" t="s">
+      <c r="E34" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="F34" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G34" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H34" s="22" t="s">
+      <c r="F34" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H34" s="21" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B35" s="11">
+      <c r="B35" s="4">
         <v>269</v>
       </c>
-      <c r="C35" s="11">
+      <c r="C35" s="4">
         <v>261</v>
       </c>
-      <c r="D35" s="11" t="s">
+      <c r="D35" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E35" s="11" t="s">
+      <c r="E35" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F35" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G35" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H35" s="13" t="s">
+      <c r="F35" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H35" s="12" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" s="21" t="s">
+      <c r="A36" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="11">
+      <c r="B36" s="4">
         <v>276</v>
       </c>
-      <c r="C36" s="11">
+      <c r="C36" s="4">
         <v>268</v>
       </c>
-      <c r="D36" s="11" t="s">
+      <c r="D36" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E36" s="11" t="s">
+      <c r="E36" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F36" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G36" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H36" s="13" t="s">
+      <c r="F36" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H36" s="12" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" s="21" t="s">
+      <c r="A37" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="4">
         <v>277</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D37" s="11" t="s">
+      <c r="D37" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E37" s="11" t="s">
+      <c r="E37" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F37" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G37" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H37" s="13" t="s">
+      <c r="F37" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H37" s="12" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A38" s="23" t="s">
+      <c r="A38" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="B38" s="16">
+      <c r="B38" s="15">
         <v>227</v>
       </c>
-      <c r="C38" s="16" t="s">
+      <c r="C38" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D38" s="16" t="s">
+      <c r="D38" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E38" s="16" t="s">
+      <c r="E38" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="F38" s="24" t="s">
+      <c r="F38" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="G38" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="H38" s="18" t="s">
+      <c r="G38" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H38" s="17" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A39" s="25" t="s">
+      <c r="A39" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B39" s="26">
+      <c r="B39" s="25">
         <v>86</v>
       </c>
-      <c r="C39" s="26">
+      <c r="C39" s="25">
         <v>85</v>
       </c>
-      <c r="D39" s="26" t="s">
+      <c r="D39" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="E39" s="26" t="s">
+      <c r="E39" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="F39" s="27" t="s">
+      <c r="F39" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="G39" s="26" t="s">
-        <v>13</v>
-      </c>
-      <c r="H39" s="28" t="s">
+      <c r="G39" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="H39" s="27" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" s="19" t="s">
+      <c r="A40" s="18" t="s">
         <v>47</v>
       </c>
       <c r="B40" s="7">
@@ -1903,210 +1910,210 @@
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41" s="21" t="s">
+      <c r="A41" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B41" s="11">
+      <c r="B41" s="4">
         <v>50</v>
       </c>
-      <c r="C41" s="11">
+      <c r="C41" s="4">
         <v>63</v>
       </c>
-      <c r="D41" s="11" t="s">
+      <c r="D41" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E41" s="11" t="s">
+      <c r="E41" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F41" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G41" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H41" s="13" t="s">
+      <c r="F41" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H41" s="12" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" s="21" t="s">
+      <c r="A42" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B42" s="11">
+      <c r="B42" s="4">
         <v>114</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D42" s="11" t="s">
+      <c r="D42" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E42" s="11" t="s">
+      <c r="E42" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F42" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G42" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H42" s="13" t="s">
+      <c r="F42" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H42" s="12" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" s="21" t="s">
+      <c r="A43" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B43" s="11">
+      <c r="B43" s="4">
         <v>129</v>
       </c>
-      <c r="C43" s="11">
+      <c r="C43" s="4">
         <v>135</v>
       </c>
-      <c r="D43" s="11" t="s">
+      <c r="D43" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E43" s="11" t="s">
+      <c r="E43" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="F43" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G43" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H43" s="13" t="s">
+      <c r="F43" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H43" s="12" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A44" s="21" t="s">
+      <c r="A44" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B44" s="11">
+      <c r="B44" s="4">
         <v>124</v>
       </c>
-      <c r="C44" s="11">
+      <c r="C44" s="4">
         <v>114</v>
       </c>
-      <c r="D44" s="11" t="s">
+      <c r="D44" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E44" s="11" t="s">
+      <c r="E44" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F44" s="12" t="s">
+      <c r="F44" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G44" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H44" s="13" t="s">
+      <c r="G44" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H44" s="12" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A45" s="21" t="s">
+      <c r="A45" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B45" s="11">
+      <c r="B45" s="4">
         <v>134</v>
       </c>
-      <c r="C45" s="11">
+      <c r="C45" s="4">
         <v>124</v>
       </c>
-      <c r="D45" s="11" t="s">
+      <c r="D45" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E45" s="11" t="s">
+      <c r="E45" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F45" s="12" t="s">
+      <c r="F45" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G45" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H45" s="13" t="s">
+      <c r="G45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H45" s="12" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A46" s="21" t="s">
+      <c r="A46" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B46" s="11">
+      <c r="B46" s="4">
         <v>138</v>
       </c>
-      <c r="C46" s="11" t="s">
+      <c r="C46" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D46" s="11" t="s">
+      <c r="D46" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E46" s="11" t="s">
+      <c r="E46" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F46" s="12" t="s">
+      <c r="F46" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G46" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H46" s="13" t="s">
+      <c r="G46" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H46" s="12" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A47" s="21" t="s">
+      <c r="A47" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B47" s="11">
+      <c r="B47" s="4">
         <v>145</v>
       </c>
-      <c r="C47" s="11">
+      <c r="C47" s="4">
         <v>135</v>
       </c>
-      <c r="D47" s="11" t="s">
+      <c r="D47" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E47" s="11" t="s">
+      <c r="E47" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="F47" s="12" t="s">
+      <c r="F47" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="G47" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H47" s="13" t="s">
+      <c r="G47" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H47" s="12" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A48" s="23" t="s">
+      <c r="A48" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="B48" s="16">
+      <c r="B48" s="15">
         <v>178</v>
       </c>
-      <c r="C48" s="16" t="s">
+      <c r="C48" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D48" s="16" t="s">
+      <c r="D48" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="E48" s="16" t="s">
+      <c r="E48" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="F48" s="24" t="s">
+      <c r="F48" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="G48" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="H48" s="18" t="s">
+      <c r="G48" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H48" s="17" t="s">
         <v>113</v>
       </c>
     </row>
@@ -2137,7 +2144,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -2146,132 +2153,140 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="C1" s="30" t="s">
+      <c r="C1" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="D1" s="30" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2" s="32" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="33" t="s">
+      <c r="A2" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="D2" s="32" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="32" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="33" t="s">
+      <c r="A3" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="32" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="35" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="36" t="s">
+      <c r="A4" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="36" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="39"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="37"/>
     </row>
     <row r="6" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="39" t="s">
         <v>60</v>
       </c>
-      <c r="C6" s="41" t="s">
+      <c r="C6" s="39" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="42" t="s">
+      <c r="D6" s="40" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="34" t="s">
         <v>117</v>
       </c>
-      <c r="C7" s="36" t="s">
+      <c r="C7" s="34" t="s">
         <v>119</v>
       </c>
-      <c r="D7" s="37" t="s">
+      <c r="D7" s="35" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="43"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="41"/>
     </row>
     <row r="9" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="D9" s="34" t="s">
+      <c r="D9" s="32" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="35" t="s">
+      <c r="A10" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="34" t="s">
         <v>120</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="C10" s="34" t="s">
         <v>119</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="D10" s="35" t="s">
         <v>43</v>
       </c>
+    </row>
+    <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="45" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" s="46"/>
+      <c r="C11" s="46"/>
+      <c r="D11" s="47"/>
     </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
@@ -2285,172 +2300,181 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="30" t="s">
+      <c r="C1" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="30" t="s">
+      <c r="D1" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="E1" s="31" t="s">
+      <c r="E1" s="30" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="32" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="33" t="s">
+      <c r="A2" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="33"/>
-      <c r="E2" s="44">
+      <c r="D2" s="3"/>
+      <c r="E2" s="42">
         <v>510</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="32" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="33" t="s">
+      <c r="A3" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="33"/>
-      <c r="E3" s="44">
+      <c r="D3" s="3"/>
+      <c r="E3" s="42">
         <v>525</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="35" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="36" t="s">
+      <c r="A4" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="36"/>
-      <c r="E4" s="45">
+      <c r="D4" s="34"/>
+      <c r="E4" s="43">
         <v>537</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="31"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="30"/>
     </row>
     <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="30"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="31"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="30"/>
     </row>
     <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="29" t="s">
+      <c r="A7" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="30"/>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="31"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="30"/>
     </row>
     <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="40" t="s">
+      <c r="A8" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="41" t="s">
+      <c r="C8" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="41"/>
-      <c r="E8" s="46">
+      <c r="D8" s="39"/>
+      <c r="E8" s="44">
         <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="33"/>
-      <c r="E9" s="44">
+      <c r="D9" s="3"/>
+      <c r="E9" s="42">
         <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="33"/>
-      <c r="E10" s="44">
+      <c r="D10" s="3"/>
+      <c r="E10" s="42">
         <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="C11" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="33"/>
-      <c r="E11" s="44">
+      <c r="D11" s="3"/>
+      <c r="E11" s="42">
         <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12" s="35" t="s">
+      <c r="A12" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="36" t="s">
+      <c r="B12" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="36" t="s">
+      <c r="C12" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="36"/>
-      <c r="E12" s="45">
+      <c r="D12" s="34"/>
+      <c r="E12" s="43">
         <v>190</v>
       </c>
+    </row>
+    <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13" s="45" t="s">
+        <v>121</v>
+      </c>
+      <c r="B13" s="46"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="46"/>
+      <c r="E13" s="47"/>
     </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
@@ -2464,7 +2488,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.1640625" style="3"/>
@@ -2473,135 +2497,144 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="30" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C2" s="44" t="s">
+      <c r="C2" s="42" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="C3" s="45" t="s">
+      <c r="C3" s="43" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="38" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="39" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="44" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="33" t="s">
         <v>78</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="45" t="s">
+      <c r="C5" s="43" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="38" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="39" t="s">
         <v>82</v>
       </c>
-      <c r="C6" s="46" t="s">
+      <c r="C6" s="44" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="34" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="45" t="s">
+      <c r="C7" s="43" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="40" t="s">
+      <c r="A8" s="38" t="s">
         <v>87</v>
       </c>
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="39" t="s">
         <v>88</v>
       </c>
-      <c r="C8" s="46" t="s">
+      <c r="C8" s="44" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C9" s="44" t="s">
+      <c r="C9" s="42" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="35" t="s">
+      <c r="A10" s="33" t="s">
         <v>93</v>
       </c>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="45" t="s">
+      <c r="C10" s="43" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="40" t="s">
+      <c r="A11" s="38" t="s">
         <v>96</v>
       </c>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="39" t="s">
         <v>97</v>
       </c>
-      <c r="C11" s="46" t="s">
+      <c r="C11" s="44" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="35" t="s">
+      <c r="A12" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="B12" s="36" t="s">
+      <c r="B12" s="34" t="s">
         <v>100</v>
       </c>
-      <c r="C12" s="45" t="s">
+      <c r="C12" s="43" t="s">
         <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="B13" s="29"/>
+      <c r="C13" s="30" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>